<commit_message>
feat: commit also study sheets and tutorial sheet
</commit_message>
<xml_diff>
--- a/example-spreadsheets/study-tasks/task-01/task01_salesCommissions.xlsx
+++ b/example-spreadsheets/study-tasks/task-01/task01_salesCommissions.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t xml:space="preserve">Task 1</t>
   </si>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t xml:space="preserve">What was the hardest part in answering these questions ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">There is an error in Levants Base Commission correct it.</t>
   </si>
 </sst>
 </file>
@@ -329,7 +332,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -383,7 +386,7 @@
         <v>10000</v>
       </c>
       <c r="D3" s="4" t="n">
-        <f aca="false">VLOOKUP(A3,A12:B18, 2, 0)</f>
+        <f aca="false">VLOOKUP(A3,$A$13:$B$18, 2, 0)</f>
         <v>0.05</v>
       </c>
       <c r="E3" s="4" t="n">
@@ -425,7 +428,7 @@
         <v>10000</v>
       </c>
       <c r="D4" s="4" t="n">
-        <f aca="false">VLOOKUP(A4,A13:B19, 2, 0)</f>
+        <f aca="false">VLOOKUP(A4,$A$13:$B$18, 2, 0)</f>
         <v>0.05</v>
       </c>
       <c r="E4" s="4" t="n">
@@ -467,7 +470,7 @@
         <v>10000</v>
       </c>
       <c r="D5" s="4" t="n">
-        <f aca="false">VLOOKUP(A5,A14:B20, 2, 0)</f>
+        <f aca="false">VLOOKUP(A5,$A$13:$B$18, 2, 0)</f>
         <v>0.03</v>
       </c>
       <c r="E5" s="4" t="n">
@@ -509,7 +512,7 @@
         <v>4200</v>
       </c>
       <c r="D6" s="4" t="n">
-        <f aca="false">VLOOKUP(A6,A15:B21, 2, 0)</f>
+        <f aca="false">VLOOKUP(A6,$A$13:$B$18, 2, 0)</f>
         <v>0.015</v>
       </c>
       <c r="E6" s="4" t="n">
@@ -551,7 +554,7 @@
         <v>8000</v>
       </c>
       <c r="D7" s="4" t="n">
-        <f aca="false">VLOOKUP(A7,A16:B22, 2, 0)</f>
+        <f aca="false">VLOOKUP(A3,$A$13:$B$18, 2, 0)</f>
         <v>0.05</v>
       </c>
       <c r="E7" s="4" t="n">
@@ -593,7 +596,7 @@
         <v>12000</v>
       </c>
       <c r="D8" s="4" t="n">
-        <f aca="false">VLOOKUP(A8,A17:B23, 2, 0)</f>
+        <f aca="false">VLOOKUP(A8,$A$13:$B$18, 2, 0)</f>
         <v>0.055</v>
       </c>
       <c r="E8" s="4" t="n">
@@ -728,6 +731,14 @@
       </c>
       <c r="B27" s="5" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>